<commit_message>
update TC AML sàng lọc
</commit_message>
<xml_diff>
--- a/.claude/skills/rbt_manual_testing/templates/TC_mau_API.xlsx
+++ b/.claude/skills/rbt_manual_testing/templates/TC_mau_API.xlsx
@@ -553,8 +553,8 @@
     <col min="4" max="4" width="11.83203125" customWidth="1"/>
     <col min="5" max="5" width="58.83203125" customWidth="1"/>
     <col min="6" max="6" width="34.83203125" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
-    <col min="8" max="8" width="48.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="34.83203125" customWidth="1"/>
     <col min="9" max="9" width="42.83203125" customWidth="1"/>
     <col min="10" max="10" width="10.83203125" customWidth="1"/>
     <col min="11" max="11" width="10.83203125" customWidth="1"/>
@@ -588,10 +588,10 @@
         <v>Pre-conditions</v>
       </c>
       <c r="G1" s="3" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="H1" s="3" t="str">
         <v>Test Data</v>
-      </c>
-      <c r="H1" s="3" t="str">
-        <v>Test Steps</v>
       </c>
       <c r="I1" s="3" t="str">
         <v>Expected result</v>
@@ -629,7 +629,7 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="str">
-        <v>NHÓM FUNCTION · BLOCK: Common · Risk: High</v>
+        <v>NHÓM FUNCTION - Common</v>
       </c>
       <c r="B2" s="4" t="str">
         <v/>
@@ -700,7 +700,7 @@
         <v>High</v>
       </c>
       <c r="E3" s="6" t="str">
-        <v>Kiểm tra gọi API thành công với Method, Token và Content-Type hợp lệ</v>
+        <v>Kiểm tra gọi API thành công với Method, Token, Content-Type và Accept header đều hợp lệ</v>
       </c>
       <c r="F3" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">- User/Quyền: Tài khoản user_a (role TRANS_REQUESTER), Bearer token_xyz còn hiệu lực
@@ -708,19 +708,16 @@
 - Dữ liệu có sẵn: Tài khoản ACC001 trạng thái Active</v>
       </c>
       <c r="G3" s="6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Gửi POST request tới API minval với Method, Token, Content-Type và Accept header đều hợp lệ (giữ nguyên data từ file minval.json).
+2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
+      </c>
+      <c r="H3" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">- Endpoint: POST https://api.sit.env/v1/trans/minval
-- Headers: Content-Type=application/json, Authorization=Bearer token_xyz
+- Headers: Content-Type=application/json, Authorization=Bearer token_xyz, Accept=application/json
 - File: minval.json
-- Body: {</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>account_id":"ACC001","amount":50000,"reason":"test"}"</v>
+- Body: {"account_id":"ACC001","amount":50000,"reason":"test"}</v>
       </c>
       <c r="I3" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Gửi POST request tới API minval với Method, Token, Content-Type header đều hợp lệ (giữ nguyên data từ file minval.json).
-2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
-      </c>
-      <c r="J3" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">2. Kiểm tra thông tin HTTP Status trả về: 200 OK
 - Json trả về có thông báo xử lý thành công: "OK"
 - Json có dạng theo format:
@@ -729,17 +726,20 @@
   "message": "OK"
 }</v>
       </c>
+      <c r="J3" s="5" t="str">
+        <v>SIT</v>
+      </c>
       <c r="K3" s="5" t="str">
-        <v>SIT</v>
+        <v>High</v>
       </c>
       <c r="L3" s="5" t="str">
-        <v>High</v>
+        <v>Yes</v>
       </c>
       <c r="M3" s="5" t="str">
         <v>Yes</v>
       </c>
       <c r="N3" s="5" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="O3" s="5" t="str">
         <v/>
@@ -754,12 +754,12 @@
         <v/>
       </c>
       <c r="S3" s="6" t="str">
-        <v/>
+        <v>TD: TD_P1_001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="str">
-        <v>NHÓM VALIDATE · BLOCK: Field 'amount' · Risk: Medium</v>
+        <v>NHÓM VALIDATE - Field 'amount'</v>
       </c>
       <c r="B4" s="4" t="str">
         <v/>
@@ -838,19 +838,16 @@
 - Dữ liệu có sẵn: Tài khoản ACC001 trạng thái Active</v>
       </c>
       <c r="G5" s="6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Gửi POST request tới API minval với body thiếu field bắt buộc 'amount'.
+2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
+      </c>
+      <c r="H5" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">- Endpoint: POST https://api.sit.env/v1/trans/minval
 - Headers: Content-Type=application/json, Authorization=Bearer token_xyz
 - File: minval.json
-- Body: {</v>
-      </c>
-      <c r="H5" s="6" t="str">
-        <v>account_id":"ACC001","amount":50000,"reason":"test"}"</v>
+- Body: {"account_id":"ACC001","reason":"test"}</v>
       </c>
       <c r="I5" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Gửi POST request tới API minval với body thiếu field bắt buộc 'amount'.
-2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
-      </c>
-      <c r="J5" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">2. Kiểm tra thông tin HTTP Status trả về: 400 Bad Request
 - Json trả về có thông báo lỗi thiếu field bắt buộc 'amount': [PENDING_DOC]
 - Json có dạng theo format:
@@ -859,17 +856,20 @@
   "message": [PENDING_DOC]
 }</v>
       </c>
+      <c r="J5" s="5" t="str">
+        <v>SIT</v>
+      </c>
       <c r="K5" s="5" t="str">
-        <v>SIT</v>
+        <v>Medium</v>
       </c>
       <c r="L5" s="5" t="str">
-        <v>High</v>
+        <v>Yes</v>
       </c>
       <c r="M5" s="5" t="str">
         <v>Yes</v>
       </c>
       <c r="N5" s="5" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="O5" s="5" t="str">
         <v/>
@@ -884,12 +884,12 @@
         <v/>
       </c>
       <c r="S5" s="6" t="str">
-        <v/>
+        <v>TD: TD_P2_004 | [PENDING_DOC] Error message chưa có trong PTTK</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="str">
-        <v>NHÓM VALIDATE · BLOCK: Giao thức HTTP · Risk: Medium</v>
+        <v>NHÓM VALIDATE - Giao thức HTTP</v>
       </c>
       <c r="B6" s="7" t="str">
         <v/>
@@ -968,19 +968,16 @@
 - Dữ liệu có sẵn: Tài khoản ACC001 trạng thái Active</v>
       </c>
       <c r="G7" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">- Endpoint: POST https://api.sit.env/v1/trans/minval
+        <v xml:space="preserve">1. Gửi POST request tới API minval với endpoint URL sai: /wrong-path/v1/trans/minval.
+2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
+      </c>
+      <c r="H7" s="6" t="str" xml:space="preserve">
+        <v xml:space="preserve">- Endpoint: POST https://api.sit.env/wrong-path/v1/trans/minval
 - Headers: Content-Type=application/json, Authorization=Bearer token_xyz
 - File: minval.json
-- Body: {</v>
-      </c>
-      <c r="H7" s="6" t="str">
-        <v>account_id":"ACC001","amount":50000,"reason":"test"}"</v>
+- Body: {"account_id":"ACC001","amount":50000,"reason":"test"}</v>
       </c>
       <c r="I7" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Gửi POST request tới API minval với endpoint URL sai: /wrong-path/v1/trans/minval.
-2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
-      </c>
-      <c r="J7" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">2. Kiểm tra thông tin HTTP Status trả về: 404 Not Found
 - Json trả về có thông báo lỗi endpoint không tồn tại: [PENDING_DOC]
 - Json có dạng theo format:
@@ -989,17 +986,20 @@
   "message": [PENDING_DOC]
 }</v>
       </c>
+      <c r="J7" s="5" t="str">
+        <v>SIT</v>
+      </c>
       <c r="K7" s="5" t="str">
-        <v>SIT</v>
+        <v>Medium</v>
       </c>
       <c r="L7" s="5" t="str">
-        <v>Medium</v>
+        <v>Yes</v>
       </c>
       <c r="M7" s="5" t="str">
         <v>Yes</v>
       </c>
       <c r="N7" s="5" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="O7" s="5" t="str">
         <v/>
@@ -1014,12 +1014,12 @@
         <v/>
       </c>
       <c r="S7" s="6" t="str">
-        <v/>
+        <v>TD: TD_P1_003 | [PENDING_DOC] Error message chưa có trong PTTK</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="str">
-        <v>NHÓM PHÂN QUYỀN · BLOCK: Authentication · Risk: High</v>
+        <v>NHÓM PHÂN QUYỀN - Authentication</v>
       </c>
       <c r="B8" s="4" t="str">
         <v/>
@@ -1090,27 +1090,24 @@
         <v>High</v>
       </c>
       <c r="E9" s="6" t="str">
-        <v>Kiểm tra API chặn truy cập thành công khi 'account_id' thuộc sở hữu của user khác</v>
+        <v>Kiểm tra API chặn truy cập thành công khi 'account_id' hợp lệ nhưng thuộc sở hữu của user khác</v>
       </c>
       <c r="F9" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">- User/Quyền: Tài khoản user_a (role TRANS_REQUESTER), Bearer token_xyz còn hiệu lực
+        <v xml:space="preserve">- User/Quyền: Tài khoản User A (role TRANS_REQUESTER), Bearer token_userA còn hiệu lực
 - Trạng thái hệ thống: Service trans-minval đang chạy trên SIT (không cần kết nối DB cho TC này)
-- Dữ liệu có sẵn: Tài khoản ACC001 trạng thái Active</v>
+- Dữ liệu có sẵn: Tài khoản ACC002 tồn tại trong DB và thuộc sở hữu của User B (không phải User A)</v>
       </c>
       <c r="G9" s="6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Gửi POST request tới API minval bằng token của User A với 'account_id' = "ACC002" (tài khoản hợp lệ nhưng thuộc sở hữu User B).
+2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
+      </c>
+      <c r="H9" s="6" t="str" xml:space="preserve">
         <v xml:space="preserve">- Endpoint: POST https://api.sit.env/v1/trans/minval
-- Headers: Content-Type=application/json, Authorization=Bearer token_xyz
+- Headers: Content-Type=application/json, Authorization=Bearer token_userA
 - File: minval.json
-- Body: {</v>
-      </c>
-      <c r="H9" s="6" t="str">
-        <v>account_id":"ACC001","amount":50000,"reason":"test"}"</v>
+- Body: {"account_id":"ACC002","amount":50000,"reason":"idor test"}</v>
       </c>
       <c r="I9" s="6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Gửi POST request tới API minval với token của User A nhưng 'account_id' = "ACC002" (tài khoản thuộc sở hữu User B).
-2. Kiểm tra thông tin HTTP Status và Response Body trả về.</v>
-      </c>
-      <c r="J9" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">2. Kiểm tra thông tin HTTP Status trả về: 403 Forbidden
 - Json trả về có thông báo từ chối truy cập tài khoản không thuộc sở hữu: [PENDING_DOC]
 - Json có dạng theo format:
@@ -1119,17 +1116,20 @@
   "message": [PENDING_DOC]
 }</v>
       </c>
+      <c r="J9" s="5" t="str">
+        <v>SIT</v>
+      </c>
       <c r="K9" s="5" t="str">
-        <v>SIT</v>
+        <v>High</v>
       </c>
       <c r="L9" s="5" t="str">
-        <v>High</v>
+        <v>Yes</v>
       </c>
       <c r="M9" s="5" t="str">
         <v>Yes</v>
       </c>
       <c r="N9" s="5" t="str">
-        <v>Yes</v>
+        <v/>
       </c>
       <c r="O9" s="5" t="str">
         <v/>
@@ -1144,7 +1144,7 @@
         <v/>
       </c>
       <c r="S9" s="6" t="str">
-        <v/>
+        <v>TD: TD_P3_013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>